<commit_message>
Renamed typologies and modified boxplots to fill by typology
</commit_message>
<xml_diff>
--- a/Copper/5. Statistical data analysis/Multiple linear regression/MLR.xlsx
+++ b/Copper/5. Statistical data analysis/Multiple linear regression/MLR.xlsx
@@ -1,85 +1,73 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
-  <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ornl-my.sharepoint.com/personal/q4q_ornl_gov/Documents/Research/Bioavailability Project/BLM_spatial_assessmt/Copper/5. Statistical data analysis/Multiple linear regression/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="19" documentId="11_C2CE303C4BA923B3705614FD1A0A53129275A262" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1F315727-3DE1-4F85-8B6F-CFC9D9ECD98B}"/>
+  <workbookPr date1904="false"/>
   <bookViews>
-    <workbookView xWindow="9510" yWindow="0" windowWidth="9780" windowHeight="11370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="13125" windowHeight="6105" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet 1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet 1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
-    <t>Predictor</t>
-  </si>
-  <si>
-    <t>Estimate</t>
-  </si>
-  <si>
-    <t>p_value</t>
-  </si>
-  <si>
-    <t>VIF</t>
-  </si>
-  <si>
-    <t>Rel_Importance</t>
-  </si>
-  <si>
-    <t>log_Cu_nM_std</t>
-  </si>
-  <si>
-    <t>pH_std</t>
-  </si>
-  <si>
-    <t>log_DOC_nM_std</t>
-  </si>
-  <si>
-    <t>log_K_nM_std</t>
-  </si>
-  <si>
-    <t>log_Na_nM_std</t>
-  </si>
-  <si>
-    <t>log_SO4_nM_std</t>
-  </si>
-  <si>
-    <t>log_Cl_nM_std</t>
-  </si>
-  <si>
-    <t>log_Ca_nM_std</t>
-  </si>
-  <si>
-    <t>log_DIC_nM_std</t>
-  </si>
-  <si>
-    <t>log_Mg_nM_std</t>
-  </si>
-  <si>
-    <t>log_Temp_C_std</t>
+    <t xml:space="preserve">Predictor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Estimate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">p_value</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VIF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rel_Importance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">log_Cu_nM_std</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pH_std</t>
+  </si>
+  <si>
+    <t xml:space="preserve">log_DOC_nM_std</t>
+  </si>
+  <si>
+    <t xml:space="preserve">log_K_nM_std</t>
+  </si>
+  <si>
+    <t xml:space="preserve">log_Na_nM_std</t>
+  </si>
+  <si>
+    <t xml:space="preserve">log_SO4_nM_std</t>
+  </si>
+  <si>
+    <t xml:space="preserve">log_Cl_nM_std</t>
+  </si>
+  <si>
+    <t xml:space="preserve">log_Ca_nM_std</t>
+  </si>
+  <si>
+    <t xml:space="preserve">log_DIC_nM_std</t>
+  </si>
+  <si>
+    <t xml:space="preserve">log_Mg_nM_std</t>
+  </si>
+  <si>
+    <t xml:space="preserve">log_Temp_C_std</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="3">
-    <numFmt numFmtId="166" formatCode="0.00000"/>
-    <numFmt numFmtId="170" formatCode="0.000"/>
-    <numFmt numFmtId="171" formatCode="0.0000"/>
-  </numFmts>
-  <fonts count="1" x14ac:knownFonts="1">
+  <numFmts count="0"/>
+  <fonts count="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -108,25 +96,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
@@ -408,14 +384,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E12"/>
-  <sheetFormatPr defaultColWidth="10.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="15.453125" bestFit="1" customWidth="1"/>
-  </cols>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -432,195 +405,195 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2">
       <c r="A2" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="1">
+      <c r="B2" t="n">
         <v>1.35672869104225</v>
       </c>
-      <c r="C2" s="2">
+      <c r="C2" t="n">
         <v>0</v>
       </c>
-      <c r="D2" s="2">
+      <c r="D2" t="n">
         <v>2.53871349901583</v>
       </c>
-      <c r="E2" s="3">
-        <v>0.62423027577812595</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E2" t="n">
+        <v>0.624230275778126</v>
+      </c>
+    </row>
+    <row r="3">
       <c r="A3" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="1">
-        <v>-0.55547549652347805</v>
-      </c>
-      <c r="C3" s="2">
-        <v>2.3473877602414698E-246</v>
-      </c>
-      <c r="D3" s="2">
-        <v>1.3937280020451699</v>
-      </c>
-      <c r="E3" s="3">
+      <c r="B3" t="n">
+        <v>-0.555475496523478</v>
+      </c>
+      <c r="C3" t="n">
+        <v>2.34738776024147e-246</v>
+      </c>
+      <c r="D3" t="n">
+        <v>1.39372800204517</v>
+      </c>
+      <c r="E3" t="n">
         <v>0.156780509182818</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="4">
       <c r="A4" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="1">
-        <v>-0.68135551174090803</v>
-      </c>
-      <c r="C4" s="2">
-        <v>1.5895996763967699E-219</v>
-      </c>
-      <c r="D4" s="2">
+      <c r="B4" t="n">
+        <v>-0.681355511740908</v>
+      </c>
+      <c r="C4" t="n">
+        <v>1.58959967639677e-219</v>
+      </c>
+      <c r="D4" t="n">
         <v>2.97837008122367</v>
       </c>
-      <c r="E4" s="3">
-        <v>9.0312686596956404E-2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E4" t="n">
+        <v>0.0903126865969564</v>
+      </c>
+    </row>
+    <row r="5">
       <c r="A5" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="1">
-        <v>-1.20258168636827E-2</v>
-      </c>
-      <c r="C5" s="2">
-        <v>0.27684250415249201</v>
-      </c>
-      <c r="D5" s="2">
-        <v>3.9631719158679402</v>
-      </c>
-      <c r="E5" s="3">
-        <v>2.8522013975922401E-2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="B5" t="n">
+        <v>-0.0120258168636827</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0.276842504152492</v>
+      </c>
+      <c r="D5" t="n">
+        <v>3.96317191586794</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.0285220139759224</v>
+      </c>
+    </row>
+    <row r="6">
       <c r="A6" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="1">
-        <v>-5.6937420739837704E-3</v>
-      </c>
-      <c r="C6" s="2">
-        <v>0.79846778762909898</v>
-      </c>
-      <c r="D6" s="2">
-        <v>16.138521052241298</v>
-      </c>
-      <c r="E6" s="3">
-        <v>2.4553492024104999E-2</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="B6" t="n">
+        <v>-0.00569374207398377</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0.798467787629099</v>
+      </c>
+      <c r="D6" t="n">
+        <v>16.1385210522413</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.024553492024105</v>
+      </c>
+    </row>
+    <row r="7">
       <c r="A7" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="1">
-        <v>4.0925748824137201E-2</v>
-      </c>
-      <c r="C7" s="2">
-        <v>2.03955563127836E-4</v>
-      </c>
-      <c r="D7" s="2">
-        <v>3.8686824629903298</v>
-      </c>
-      <c r="E7" s="3">
-        <v>2.3903693275118099E-2</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="B7" t="n">
+        <v>0.0409257488241372</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0.000203955563127836</v>
+      </c>
+      <c r="D7" t="n">
+        <v>3.86868246299033</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.0239036932751181</v>
+      </c>
+    </row>
+    <row r="8">
       <c r="A8" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="1">
-        <v>-4.7190127166013798E-2</v>
-      </c>
-      <c r="C8" s="2">
-        <v>6.1215429878439497E-3</v>
-      </c>
-      <c r="D8" s="2">
+      <c r="B8" t="n">
+        <v>-0.0471901271660138</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0.00612154298784395</v>
+      </c>
+      <c r="D8" t="n">
         <v>9.52265199934725</v>
       </c>
-      <c r="E8" s="3">
-        <v>1.6693382718024698E-2</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E8" t="n">
+        <v>0.0166933827180247</v>
+      </c>
+    </row>
+    <row r="9">
       <c r="A9" t="s">
         <v>12</v>
       </c>
-      <c r="B9" s="1">
-        <v>-2.3706571606703499E-2</v>
-      </c>
-      <c r="C9" s="2">
-        <v>0.15816144783532601</v>
-      </c>
-      <c r="D9" s="2">
+      <c r="B9" t="n">
+        <v>-0.0237065716067035</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0.158161447835326</v>
+      </c>
+      <c r="D9" t="n">
         <v>9.13404853479142</v>
       </c>
-      <c r="E9" s="3">
-        <v>1.29797927329226E-2</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E9" t="n">
+        <v>0.0129797927329226</v>
+      </c>
+    </row>
+    <row r="10">
       <c r="A10" t="s">
         <v>13</v>
       </c>
-      <c r="B10" s="1">
-        <v>-1.40980592137172E-2</v>
-      </c>
-      <c r="C10" s="2">
-        <v>0.39116479192645898</v>
-      </c>
-      <c r="D10" s="2">
-        <v>8.7645093383482209</v>
-      </c>
-      <c r="E10" s="1">
-        <v>8.0940627015919295E-3</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="B10" t="n">
+        <v>-0.0140980592137172</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0.391164791926459</v>
+      </c>
+      <c r="D10" t="n">
+        <v>8.76450933834822</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.00809406270159193</v>
+      </c>
+    </row>
+    <row r="11">
       <c r="A11" t="s">
         <v>14</v>
       </c>
-      <c r="B11" s="1">
-        <v>-1.3057284900288801E-2</v>
-      </c>
-      <c r="C11" s="2">
-        <v>0.28472077580900901</v>
-      </c>
-      <c r="D11" s="2">
-        <v>4.8280028331817002</v>
-      </c>
-      <c r="E11" s="1">
-        <v>7.6696592037478802E-3</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="B11" t="n">
+        <v>-0.0130572849002888</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0.284720775809009</v>
+      </c>
+      <c r="D11" t="n">
+        <v>4.8280028331817</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0.00766965920374788</v>
+      </c>
+    </row>
+    <row r="12">
       <c r="A12" t="s">
         <v>15</v>
       </c>
-      <c r="B12" s="1">
-        <v>-5.1092098784435998E-2</v>
-      </c>
-      <c r="C12" s="2">
-        <v>7.7952006397846298E-16</v>
-      </c>
-      <c r="D12" s="2">
+      <c r="B12" t="n">
+        <v>-0.051092098784436</v>
+      </c>
+      <c r="C12" t="n">
+        <v>0.000000000000000779520063978463</v>
+      </c>
+      <c r="D12" t="n">
         <v>1.19495270731042</v>
       </c>
-      <c r="E12" s="1">
-        <v>6.2604318106673704E-3</v>
+      <c r="E12" t="n">
+        <v>0.00626043181066737</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Compared full MLR to a simplified MLR to predict Zn and Cu bioavail
</commit_message>
<xml_diff>
--- a/Copper/5. Statistical data analysis/Multiple linear regression/MLR.xlsx
+++ b/Copper/5. Statistical data analysis/Multiple linear regression/MLR.xlsx
@@ -38,12 +38,12 @@
     <t xml:space="preserve">log_DOC_nM_std</t>
   </si>
   <si>
+    <t xml:space="preserve">log_Na_nM_std</t>
+  </si>
+  <si>
     <t xml:space="preserve">log_K_nM_std</t>
   </si>
   <si>
-    <t xml:space="preserve">log_Na_nM_std</t>
-  </si>
-  <si>
     <t xml:space="preserve">log_SO4_nM_std</t>
   </si>
   <si>
@@ -53,13 +53,13 @@
     <t xml:space="preserve">log_Ca_nM_std</t>
   </si>
   <si>
+    <t xml:space="preserve">log_Temp_C_std</t>
+  </si>
+  <si>
     <t xml:space="preserve">log_DIC_nM_std</t>
   </si>
   <si>
     <t xml:space="preserve">log_Mg_nM_std</t>
-  </si>
-  <si>
-    <t xml:space="preserve">log_Temp_C_std</t>
   </si>
 </sst>
 </file>
@@ -410,16 +410,16 @@
         <v>5</v>
       </c>
       <c r="B2" t="n">
-        <v>1.35672869104225</v>
+        <v>1.34720729087859</v>
       </c>
       <c r="C2" t="n">
-        <v>0</v>
+        <v>1.93382755337073e-312</v>
       </c>
       <c r="D2" t="n">
-        <v>2.53871349901583</v>
+        <v>2.54560775861302</v>
       </c>
       <c r="E2" t="n">
-        <v>0.624230275778126</v>
+        <v>0.627087283938181</v>
       </c>
     </row>
     <row r="3">
@@ -427,16 +427,16 @@
         <v>6</v>
       </c>
       <c r="B3" t="n">
-        <v>-0.555475496523478</v>
+        <v>-0.53074332141694</v>
       </c>
       <c r="C3" t="n">
-        <v>2.34738776024147e-246</v>
+        <v>7.88771978470265e-219</v>
       </c>
       <c r="D3" t="n">
-        <v>1.39372800204517</v>
+        <v>1.44064520760624</v>
       </c>
       <c r="E3" t="n">
-        <v>0.156780509182818</v>
+        <v>0.147820642405235</v>
       </c>
     </row>
     <row r="4">
@@ -444,16 +444,16 @@
         <v>7</v>
       </c>
       <c r="B4" t="n">
-        <v>-0.681355511740908</v>
+        <v>-0.655259618119645</v>
       </c>
       <c r="C4" t="n">
-        <v>1.58959967639677e-219</v>
+        <v>0.000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000000780422424244998</v>
       </c>
       <c r="D4" t="n">
-        <v>2.97837008122367</v>
+        <v>2.79835401362034</v>
       </c>
       <c r="E4" t="n">
-        <v>0.0903126865969564</v>
+        <v>0.0906589436958603</v>
       </c>
     </row>
     <row r="5">
@@ -461,16 +461,16 @@
         <v>8</v>
       </c>
       <c r="B5" t="n">
-        <v>-0.0120258168636827</v>
+        <v>-0.0026221572434501</v>
       </c>
       <c r="C5" t="n">
-        <v>0.276842504152492</v>
+        <v>0.917504985883087</v>
       </c>
       <c r="D5" t="n">
-        <v>3.96317191586794</v>
+        <v>19.3699009872279</v>
       </c>
       <c r="E5" t="n">
-        <v>0.0285220139759224</v>
+        <v>0.0290517929260689</v>
       </c>
     </row>
     <row r="6">
@@ -478,16 +478,16 @@
         <v>9</v>
       </c>
       <c r="B6" t="n">
-        <v>-0.00569374207398377</v>
+        <v>-0.0120736553164605</v>
       </c>
       <c r="C6" t="n">
-        <v>0.798467787629099</v>
+        <v>0.345758948602271</v>
       </c>
       <c r="D6" t="n">
-        <v>16.1385210522413</v>
+        <v>4.94967528991723</v>
       </c>
       <c r="E6" t="n">
-        <v>0.024553492024105</v>
+        <v>0.0285636618933346</v>
       </c>
     </row>
     <row r="7">
@@ -495,16 +495,16 @@
         <v>10</v>
       </c>
       <c r="B7" t="n">
-        <v>0.0409257488241372</v>
+        <v>0.032441084846519</v>
       </c>
       <c r="C7" t="n">
-        <v>0.000203955563127836</v>
+        <v>0.00557440539491165</v>
       </c>
       <c r="D7" t="n">
-        <v>3.86868246299033</v>
+        <v>4.0939287415833</v>
       </c>
       <c r="E7" t="n">
-        <v>0.0239036932751181</v>
+        <v>0.024317369731219</v>
       </c>
     </row>
     <row r="8">
@@ -512,16 +512,16 @@
         <v>11</v>
       </c>
       <c r="B8" t="n">
-        <v>-0.0471901271660138</v>
+        <v>-0.034214480669279</v>
       </c>
       <c r="C8" t="n">
-        <v>0.00612154298784395</v>
+        <v>0.0648337866635752</v>
       </c>
       <c r="D8" t="n">
-        <v>9.52265199934725</v>
+        <v>10.3265365918509</v>
       </c>
       <c r="E8" t="n">
-        <v>0.0166933827180247</v>
+        <v>0.018892922623952</v>
       </c>
     </row>
     <row r="9">
@@ -529,16 +529,16 @@
         <v>12</v>
       </c>
       <c r="B9" t="n">
-        <v>-0.0237065716067035</v>
+        <v>-0.0295168823648154</v>
       </c>
       <c r="C9" t="n">
-        <v>0.158161447835326</v>
+        <v>0.0844451331890632</v>
       </c>
       <c r="D9" t="n">
-        <v>9.13404853479142</v>
+        <v>8.80630321544478</v>
       </c>
       <c r="E9" t="n">
-        <v>0.0129797927329226</v>
+        <v>0.0110393607655796</v>
       </c>
     </row>
     <row r="10">
@@ -546,16 +546,16 @@
         <v>13</v>
       </c>
       <c r="B10" t="n">
-        <v>-0.0140980592137172</v>
+        <v>-0.0552551142818269</v>
       </c>
       <c r="C10" t="n">
-        <v>0.391164791926459</v>
+        <v>0.000000000000000250562692550019</v>
       </c>
       <c r="D10" t="n">
-        <v>8.76450933834822</v>
+        <v>1.24409781629897</v>
       </c>
       <c r="E10" t="n">
-        <v>0.00809406270159193</v>
+        <v>0.00941936334920962</v>
       </c>
     </row>
     <row r="11">
@@ -563,16 +563,16 @@
         <v>14</v>
       </c>
       <c r="B11" t="n">
-        <v>-0.0130572849002888</v>
+        <v>-0.0013580035556857</v>
       </c>
       <c r="C11" t="n">
-        <v>0.284720775809009</v>
+        <v>0.935259212217569</v>
       </c>
       <c r="D11" t="n">
-        <v>4.8280028331817</v>
+        <v>8.44716511552504</v>
       </c>
       <c r="E11" t="n">
-        <v>0.00766965920374788</v>
+        <v>0.00668730036121604</v>
       </c>
     </row>
     <row r="12">
@@ -580,16 +580,16 @@
         <v>15</v>
       </c>
       <c r="B12" t="n">
-        <v>-0.051092098784436</v>
+        <v>-0.0288792080868142</v>
       </c>
       <c r="C12" t="n">
-        <v>0.000000000000000779520063978463</v>
+        <v>0.020075592105186</v>
       </c>
       <c r="D12" t="n">
-        <v>1.19495270731042</v>
+        <v>4.62672094846105</v>
       </c>
       <c r="E12" t="n">
-        <v>0.00626043181066737</v>
+        <v>0.00646135831014396</v>
       </c>
     </row>
   </sheetData>

</xml_diff>